<commit_message>
perf: opt xlsx tool
</commit_message>
<xml_diff>
--- a/game_conf/xls/枚举@enum.xlsx
+++ b/game_conf/xls/枚举@enum.xlsx
@@ -1,64 +1,39 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
-  <workbookPr filterPrivacy="true" defaultThemeVersion="164011"/>
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <workbookPr/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="14805" windowHeight="8010"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="28680" yWindow="-120" windowWidth="16440" windowHeight="28320" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="枚举表@enum" sheetId="1" r:id="rId1"/>
-    <sheet name="生成表" sheetId="2" r:id="rId5"/>
+    <sheet name="枚举表@enum" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="生成表" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
-  <calcPr calcId="122211"/>
+  <definedNames/>
+  <calcPr calcId="122211" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
-<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="9" uniqueCount="9">
-  <si>
-    <t>E|道具类型-空|PropertyType|Empty|0</t>
-  </si>
-  <si>
-    <t>E|品质类型-空|QualityType|None|0</t>
-  </si>
-  <si>
-    <t>E|任务类型-空|TaskType|NONE|0</t>
-  </si>
-  <si>
-    <t>E|道具类型-金币|PropertyType|Coin|1</t>
-  </si>
-  <si>
-    <t>E|品质类型-白|QualityType|White|1</t>
-  </si>
-  <si>
-    <t>E|任务类型-主线|TaskType|MAIN|1</t>
-  </si>
-  <si>
-    <t>E|道具类型-钻石|PropertyType|Diamond|2</t>
-  </si>
-  <si>
-    <t>E|品质类型-蓝|QualityType|Blue|2</t>
-  </si>
-  <si>
-    <t>@enum|枚举表@enum</t>
-  </si>
-</sst>
-</file>
-
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:ap="http://schemas.openxmlformats.org/officeDocument/2006/extended-properties" xmlns:op="http://schemas.openxmlformats.org/officeDocument/2006/custom-properties" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:cdr="http://schemas.openxmlformats.org/drawingml/2006/chartDrawing" xmlns:comp="http://schemas.openxmlformats.org/drawingml/2006/compatibility" xmlns:dgm="http://schemas.openxmlformats.org/drawingml/2006/diagram" xmlns:lc="http://schemas.openxmlformats.org/drawingml/2006/lockedCanvas" xmlns:pic="http://schemas.openxmlformats.org/drawingml/2006/picture" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" xmlns:m="http://schemas.openxmlformats.org/officeDocument/2006/math" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:sl="http://schemas.openxmlformats.org/schemaLibrary/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xne="http://schemas.microsoft.com/office/excel/2006/main" xmlns:mso="http://schemas.microsoft.com/office/2006/01/customui" xmlns:ax="http://schemas.microsoft.com/office/2006/activeX" xmlns:cppr="http://schemas.microsoft.com/office/2006/coverPageProps" xmlns:cdip="http://schemas.microsoft.com/office/2006/customDocumentInformationPanel" xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ntns="http://schemas.microsoft.com/office/2006/metadata/customXsn" xmlns:lp="http://schemas.microsoft.com/office/2006/metadata/longProperties" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" xmlns:msink="http://schemas.microsoft.com/ink/2010/main" xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" xmlns:cdr14="http://schemas.microsoft.com/office/drawing/2010/chartDrawing" xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" xmlns:pic14="http://schemas.microsoft.com/office/drawing/2010/picture" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xdr14="http://schemas.microsoft.com/office/excel/2010/spreadsheetDrawing" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:dsp="http://schemas.microsoft.com/office/drawing/2008/diagram" xmlns:mso14="http://schemas.microsoft.com/office/2009/07/customui" xmlns:dgm14="http://schemas.microsoft.com/office/drawing/2010/diagram" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:x12ac="http://schemas.microsoft.com/office/spreadsheetml/2011/1/ac" xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" xmlns:xr4="http://schemas.microsoft.com/office/spreadsheetml/2016/revision4" xmlns:xr5="http://schemas.microsoft.com/office/spreadsheetml/2016/revision5" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr7="http://schemas.microsoft.com/office/spreadsheetml/2016/revision7" xmlns:xr8="http://schemas.microsoft.com/office/spreadsheetml/2016/revision8" xmlns:xr9="http://schemas.microsoft.com/office/spreadsheetml/2016/revision9" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr11="http://schemas.microsoft.com/office/spreadsheetml/2016/revision11" xmlns:xr12="http://schemas.microsoft.com/office/spreadsheetml/2016/revision12" xmlns:xr13="http://schemas.microsoft.com/office/spreadsheetml/2016/revision13" xmlns:xr14="http://schemas.microsoft.com/office/spreadsheetml/2016/revision14" xmlns:xr15="http://schemas.microsoft.com/office/spreadsheetml/2016/revision15" xmlns:x16="http://schemas.microsoft.com/office/spreadsheetml/2014/11/main" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:mo="http://schemas.microsoft.com/office/mac/office/2008/main" xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" xmlns:mv="urn:schemas-microsoft-com:mac:vml" xmlns:o="urn:schemas-microsoft-com:office:office" xmlns:v="urn:schemas-microsoft-com:vml" mc:Ignorable="c14 cdr14 a14 pic14 x14 xdr14 x14ac dsp mso14 dgm14 x15 x12ac x15ac xr xr2 xr3 xr4 xr5 xr6 xr7 xr8 xr9 xr10 xr11 xr12 xr13 xr14 xr15 x15 x16 x16r2 mo mx mv o v" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <fonts count="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <numFmts count="0"/>
+  <fonts count="2">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
     </font>
+    <font>
+      <name val="宋体"/>
+      <charset val="134"/>
+      <family val="3"/>
+      <sz val="9"/>
+    </font>
   </fonts>
   <fills count="2">
     <fill>
-      <patternFill patternType="none"/>
+      <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
@@ -77,18 +52,85 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
   <cellXfs count="1">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="0"/>
-  <tableStyles count="0" defaultPivotStyle="PivotStyleLight16" defaultTableStyle="TableStyleMedium2"/>
+  <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
+  <colors>
+    <indexedColors>
+      <rgbColor rgb="00000000"/>
+      <rgbColor rgb="00FFFFFF"/>
+      <rgbColor rgb="00FF0000"/>
+      <rgbColor rgb="0000FF00"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00000000"/>
+      <rgbColor rgb="00FFFFFF"/>
+      <rgbColor rgb="00FF0000"/>
+      <rgbColor rgb="0000FF00"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00800000"/>
+      <rgbColor rgb="00008000"/>
+      <rgbColor rgb="00000080"/>
+      <rgbColor rgb="00808000"/>
+      <rgbColor rgb="00800080"/>
+      <rgbColor rgb="00008080"/>
+      <rgbColor rgb="00C0C0C0"/>
+      <rgbColor rgb="00808080"/>
+      <rgbColor rgb="009999FF"/>
+      <rgbColor rgb="00993366"/>
+      <rgbColor rgb="00FFFFCC"/>
+      <rgbColor rgb="00CCFFFF"/>
+      <rgbColor rgb="00660066"/>
+      <rgbColor rgb="00FF8080"/>
+      <rgbColor rgb="000066CC"/>
+      <rgbColor rgb="00CCCCFF"/>
+      <rgbColor rgb="00000080"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00800080"/>
+      <rgbColor rgb="00800000"/>
+      <rgbColor rgb="00008080"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="0000CCFF"/>
+      <rgbColor rgb="00CCFFFF"/>
+      <rgbColor rgb="00CCFFCC"/>
+      <rgbColor rgb="00FFFF99"/>
+      <rgbColor rgb="0099CCFF"/>
+      <rgbColor rgb="00FF99CC"/>
+      <rgbColor rgb="00CC99FF"/>
+      <rgbColor rgb="00FFCC99"/>
+      <rgbColor rgb="003366FF"/>
+      <rgbColor rgb="0033CCCC"/>
+      <rgbColor rgb="0099CC00"/>
+      <rgbColor rgb="00FFCC00"/>
+      <rgbColor rgb="00FF9900"/>
+      <rgbColor rgb="00FF6600"/>
+      <rgbColor rgb="00666699"/>
+      <rgbColor rgb="00969696"/>
+      <rgbColor rgb="00003366"/>
+      <rgbColor rgb="00339966"/>
+      <rgbColor rgb="00003300"/>
+      <rgbColor rgb="00333300"/>
+      <rgbColor rgb="00993300"/>
+      <rgbColor rgb="00993366"/>
+      <rgbColor rgb="00333399"/>
+      <rgbColor rgb="00333333"/>
+    </indexedColors>
+  </colors>
 </styleSheet>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
   <a:themeElements>
     <a:clrScheme name="Office">
       <a:dk1>
@@ -344,53 +386,82 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:C3"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" t="s">
-        <v>2</v>
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>E|道具类型-空|PropertyType|Empty|0</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>E|品质类型-空|QualityType|None|0</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>E|任务类型-空|TaskType|NONE|0</t>
+        </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="s">
-        <v>3</v>
-      </c>
-      <c r="B2" t="s">
-        <v>4</v>
-      </c>
-      <c r="C2" t="s">
-        <v>5</v>
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>E|道具类型-金币|PropertyType|Coin|1</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>E|品质类型-白|QualityType|White|1</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>E|任务类型-主线|TaskType|MAIN|1</t>
+        </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" t="s">
-        <v>6</v>
-      </c>
-      <c r="B3" t="s">
-        <v>7</v>
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>E|道具类型-钻石|PropertyType|Diamond|2</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>E|品质类型-蓝|QualityType|Blue|2</t>
+        </is>
       </c>
     </row>
   </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1"/>
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:B1"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" t="s">
-        <v>8</v>
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>@enum|枚举表@enum</t>
+        </is>
       </c>
     </row>
   </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>